<commit_message>
Adopt the new assignments: figures, tables, methods and prose
Figure 4, Figure S6, and Tables S9, S10, S11, S15, S16 copied from the code
repo. The methods give the new mSigAct routing rule with counts from
ms_numbers.R. The sex-bias and age paragraphs follow the new Tables S15
and S16. The blue Table S11 note, CLAUDE.md and paper_to_do.md are updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EJGU7D6hCyhVnYFFhku6cJ
</commit_message>
<xml_diff>
--- a/sup_tables/sup_table_s10_insdel_N_burden.xlsx
+++ b/sup_tables/sup_table_s10_insdel_N_burden.xlsx
@@ -171,22 +171,22 @@
     <t xml:space="preserve">CPCT02340022T</t>
   </si>
   <si>
+    <t xml:space="preserve">DRUP01070119T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP16886</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02220023T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRUP01010108T</t>
+  </si>
+  <si>
     <t xml:space="preserve">SP105018</t>
   </si>
   <si>
-    <t xml:space="preserve">DRUP01070119T</t>
-  </si>
-  <si>
     <t xml:space="preserve">SP19295</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP16886</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02220023T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRUP01010108T</t>
   </si>
 </sst>
 </file>
@@ -627,16 +627,16 @@
         <v>100</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>1790</v>
+        <v>1830</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>1286</v>
+        <v>1315</v>
       </c>
       <c r="G4" s="5" t="n">
         <v>2</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>10903</v>
+        <v>21806</v>
       </c>
     </row>
     <row r="5">
@@ -647,22 +647,22 @@
         <v>12</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.81</v>
+        <v>0.89</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>521</v>
+        <v>731</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>252</v>
+        <v>428</v>
       </c>
       <c r="G5" s="5" t="n">
         <v>8</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>3344</v>
+        <v>3396</v>
       </c>
     </row>
     <row r="6">
@@ -673,22 +673,22 @@
         <v>13</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>2629</v>
+        <v>2409</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>38.83</v>
+        <v>35.58</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>2514</v>
+        <v>2553</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>2098</v>
+        <v>2118</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>9414</v>
+        <v>9416</v>
       </c>
     </row>
     <row r="7">
@@ -699,22 +699,22 @@
         <v>14</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>1312</v>
+        <v>1272</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>19.38</v>
+        <v>18.79</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>2743</v>
+        <v>2727</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>2303</v>
+        <v>2301</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>9414</v>
+        <v>9134</v>
       </c>
     </row>
     <row r="8">
@@ -725,16 +725,16 @@
         <v>15</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>1187</v>
+        <v>1022</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>17.53</v>
+        <v>15.1</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>2371</v>
+        <v>2413</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>2010</v>
+        <v>2015</v>
       </c>
       <c r="G8" s="5" t="n">
         <v>130</v>
@@ -751,22 +751,22 @@
         <v>16</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>1.92</v>
+        <v>1.7</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>1515</v>
+        <v>1868</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>1030</v>
+        <v>1210</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>180</v>
+        <v>246</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>6716</v>
+        <v>9416</v>
       </c>
     </row>
     <row r="10">
@@ -777,22 +777,22 @@
         <v>17</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>2596</v>
+        <v>2724</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>38.35</v>
+        <v>40.24</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1330</v>
+        <v>1415</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>1026</v>
+        <v>1088</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>8906</v>
+        <v>16622</v>
       </c>
     </row>
     <row r="11">
@@ -819,16 +819,16 @@
         <v>100</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>57474</v>
+        <v>114948</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>39284</v>
+        <v>78564</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>3876</v>
+        <v>7752</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>267487</v>
+        <v>534972</v>
       </c>
     </row>
     <row r="13">
@@ -845,16 +845,16 @@
         <v>1.14</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>12631</v>
+        <v>84454</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>12631</v>
+        <v>84454</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>5164</v>
+        <v>10332</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>20098</v>
+        <v>158576</v>
       </c>
     </row>
     <row r="14">
@@ -865,22 +865,22 @@
         <v>13</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>5.14</v>
+        <v>5.71</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>6973</v>
+        <v>13135</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>4854</v>
+        <v>8758</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>4261</v>
+        <v>7752</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>20098</v>
+        <v>40198</v>
       </c>
     </row>
     <row r="15">
@@ -891,22 +891,22 @@
         <v>14</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>3.43</v>
+        <v>2.86</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>4517</v>
+        <v>8566</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>4379</v>
+        <v>8522</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>4261</v>
+        <v>7752</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>4937</v>
+        <v>9878</v>
       </c>
     </row>
     <row r="16">
@@ -917,22 +917,22 @@
         <v>15</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>0.57</v>
+        <v>1.14</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>6171</v>
+        <v>10462</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>6171</v>
+        <v>10462</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>6171</v>
+        <v>8582</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>6171</v>
+        <v>12342</v>
       </c>
     </row>
     <row r="17">
@@ -943,22 +943,22 @@
         <v>16</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>1.14</v>
+        <v>1.71</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>14741</v>
+        <v>22533</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>14741</v>
+        <v>18770</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>9384</v>
+        <v>8632</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>20098</v>
+        <v>40198</v>
       </c>
     </row>
     <row r="18">
@@ -969,22 +969,22 @@
         <v>17</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>20</v>
+        <v>23.43</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>28690</v>
+        <v>76586</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>7721</v>
+        <v>29242</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>3876</v>
+        <v>8098</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>115376</v>
+        <v>534972</v>
       </c>
     </row>
   </sheetData>
@@ -1052,7 +1052,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>208437</v>
+        <v>416874</v>
       </c>
       <c r="E3" s="8" t="n">
         <v>0</v>
@@ -1072,7 +1072,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>204296</v>
+        <v>408590</v>
       </c>
       <c r="E4" s="8" t="n">
         <v>0</v>
@@ -1092,7 +1092,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>162233</v>
+        <v>324464</v>
       </c>
       <c r="E5" s="8" t="n">
         <v>0</v>
@@ -1112,7 +1112,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>160870</v>
+        <v>321738</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>0</v>
@@ -1132,7 +1132,7 @@
         <v>1</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>160618</v>
+        <v>321236</v>
       </c>
       <c r="E7" s="8" t="n">
         <v>0</v>
@@ -1152,7 +1152,7 @@
         <v>1</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>153646</v>
+        <v>307292</v>
       </c>
       <c r="E8" s="8" t="n">
         <v>0</v>
@@ -1172,7 +1172,7 @@
         <v>1</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>133385</v>
+        <v>266770</v>
       </c>
       <c r="E9" s="8" t="n">
         <v>0</v>
@@ -1192,10 +1192,10 @@
         <v>1</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>129339</v>
+        <v>258680</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>107027</v>
+        <v>186680</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>0</v>
@@ -1212,10 +1212,10 @@
         <v>1</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>127212</v>
+        <v>254424</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>98181</v>
+        <v>206824</v>
       </c>
       <c r="F11" s="8" t="n">
         <v>0</v>
@@ -1232,7 +1232,7 @@
         <v>1</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>126973</v>
+        <v>253948</v>
       </c>
       <c r="E12" s="8" t="n">
         <v>0</v>
@@ -1252,7 +1252,7 @@
         <v>1</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>126071</v>
+        <v>252144</v>
       </c>
       <c r="E13" s="8" t="n">
         <v>0</v>
@@ -1272,7 +1272,7 @@
         <v>1</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>110596</v>
+        <v>221192</v>
       </c>
       <c r="E14" s="8" t="n">
         <v>0</v>
@@ -1292,7 +1292,7 @@
         <v>1</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>105183</v>
+        <v>210364</v>
       </c>
       <c r="E15" s="8" t="n">
         <v>0</v>
@@ -1312,7 +1312,7 @@
         <v>1</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>95879</v>
+        <v>191760</v>
       </c>
       <c r="E16" s="8" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
         <v>1</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>29442</v>
+        <v>58880</v>
       </c>
       <c r="E17" s="8" t="n">
         <v>0</v>
@@ -1352,10 +1352,10 @@
         <v>1</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>29055</v>
+        <v>58110</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>3271</v>
+        <v>9112</v>
       </c>
       <c r="F18" s="8" t="n">
         <v>0</v>
@@ -1372,7 +1372,7 @@
         <v>1</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>25666</v>
+        <v>51334</v>
       </c>
       <c r="E19" s="8" t="n">
         <v>0</v>
@@ -1392,7 +1392,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>19338</v>
+        <v>38678</v>
       </c>
       <c r="E20" s="8" t="n">
         <v>0</v>
@@ -1412,10 +1412,10 @@
         <v>1</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>16801</v>
+        <v>33600</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>2934</v>
+        <v>7908</v>
       </c>
       <c r="F21" s="8" t="n">
         <v>0</v>
@@ -1432,7 +1432,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>15129</v>
+        <v>30260</v>
       </c>
       <c r="E22" s="8" t="n">
         <v>0</v>
@@ -1452,7 +1452,7 @@
         <v>1</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>14578</v>
+        <v>29158</v>
       </c>
       <c r="E23" s="8" t="n">
         <v>0</v>
@@ -1472,10 +1472,10 @@
         <v>1</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>11589</v>
+        <v>23178</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>0</v>
+        <v>2768</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>0</v>
@@ -1492,7 +1492,7 @@
         <v>1</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>10551</v>
+        <v>21104</v>
       </c>
       <c r="E25" s="8" t="n">
         <v>0</v>
@@ -1512,7 +1512,7 @@
         <v>1</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>10369</v>
+        <v>20738</v>
       </c>
       <c r="E26" s="8" t="n">
         <v>0</v>
@@ -1529,13 +1529,13 @@
         <v>26</v>
       </c>
       <c r="C27" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>9414</v>
+        <v>17800</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>924</v>
+        <v>0</v>
       </c>
       <c r="F27" s="8" t="n">
         <v>0</v>
@@ -1546,13 +1546,13 @@
         <v>53</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C28" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>8900</v>
+        <v>15324</v>
       </c>
       <c r="E28" s="8" t="n">
         <v>0</v>
@@ -1566,19 +1566,19 @@
         <v>54</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C29" s="4" t="b">
         <v>0</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>8556</v>
+        <v>12722</v>
       </c>
       <c r="E29" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>2987</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -1586,19 +1586,19 @@
         <v>55</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C30" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>7663</v>
+        <v>10828</v>
       </c>
       <c r="E30" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>0</v>
+        <v>5228</v>
       </c>
     </row>
     <row r="31">
@@ -1612,7 +1612,7 @@
         <v>0</v>
       </c>
       <c r="D31" s="8" t="n">
-        <v>6361</v>
+        <v>9414</v>
       </c>
       <c r="E31" s="8" t="n">
         <v>0</v>
@@ -1626,19 +1626,19 @@
         <v>57</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C32" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>5415</v>
+        <v>8554</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>0</v>
+        <v>810</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>4018</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New MSI-H calls (204): Figure 4, Tables S9, S10, S16 (code repo a91522c, data repo 19c3508); CLAUDE.md, paper_to_do, data_flow
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BtpRPVo656vetvDm7bkL5X
</commit_message>
<xml_diff>
--- a/sup_tables/sup_table_s10_insdel_N_burden.xlsx
+++ b/sup_tables/sup_table_s10_insdel_N_burden.xlsx
@@ -15,7 +15,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
-    <t xml:space="preserve">Table S10, Signature InsDel_N_alpha and InsDel_N_beta burden by MSI status and in conjunction with InsDel1a/1b/1c mutations. Any: All analyzed tumors of that MSI status, whatever signatures they carry. This row is the reference for the rows below it. Overlapping categories: The four InsDel1-family rows dissect co-occurrence with InsDel_N_beta and are not disjoint. A tumor with InsDel_N_beta, InsDel1a and InsDel1b is counted in both the 'and InsDel1a' and the 'and InsDel1b/1c' rows. Tumors analyzed: 6945 of 6975 (175 MSI-H, 6770 MSS). Source data: liu_et_al_89_assignment.tsv and sample_info.tsv from https://github.com/indelsig/unified_indels_data/. Generated by: build_sup_table_s10/build_sup_table_s10.R.</t>
+    <t xml:space="preserve">Table S10, Signature InsDel_N_alpha and InsDel_N_beta burden by MSI status and in conjunction with InsDel1a/1b/1c mutations. Any: All analyzed tumors of that MSI status, whatever signatures they carry. This row is the reference for the rows below it. Overlapping categories: The four InsDel1-family rows dissect co-occurrence with InsDel_N_beta and are not disjoint. A tumor with InsDel_N_beta, InsDel1a and InsDel1b is counted in both the 'and InsDel1a' and the 'and InsDel1b/1c' rows. Tumors analyzed: 6945 of 6975 (177 MSI-H, 6768 MSS). Source data: liu_et_al_89_assignment.tsv and sample_info.tsv from https://github.com/indelsig/unified_indels_data/. Generated by: build_sup_table_s10/build_sup_table_s10.R.</t>
   </si>
   <si>
     <t xml:space="preserve">MSI status</t>
@@ -621,16 +621,16 @@
         <v>11</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>6770</v>
+        <v>6768</v>
       </c>
       <c r="D4" s="7" t="n">
         <v>100</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>1830</v>
+        <v>1833</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="G4" s="5" t="n">
         <v>2</v>
@@ -673,16 +673,16 @@
         <v>13</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>2409</v>
+        <v>2403</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>35.58</v>
+        <v>35.51</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>2553</v>
+        <v>2539</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>2118</v>
+        <v>2110</v>
       </c>
       <c r="G6" s="5" t="n">
         <v>28</v>
@@ -699,22 +699,22 @@
         <v>14</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>1272</v>
+        <v>1267</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>18.79</v>
+        <v>18.72</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>2727</v>
+        <v>2705</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>2301</v>
+        <v>2294</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>28</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>9134</v>
+        <v>7992</v>
       </c>
     </row>
     <row r="8">
@@ -725,22 +725,22 @@
         <v>15</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>15.1</v>
+        <v>15.09</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>2413</v>
+        <v>2408</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="G8" s="5" t="n">
         <v>130</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>7928</v>
+        <v>7794</v>
       </c>
     </row>
     <row r="9">
@@ -777,13 +777,13 @@
         <v>17</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>2724</v>
+        <v>2726</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>40.24</v>
+        <v>40.28</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1415</v>
+        <v>1425</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>1088</v>
@@ -813,19 +813,19 @@
         <v>11</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D12" s="7" t="n">
         <v>100</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>114948</v>
+        <v>113578</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>78564</v>
+        <v>78536</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>7752</v>
+        <v>7700</v>
       </c>
       <c r="H12" s="5" t="n">
         <v>534972</v>
@@ -842,7 +842,7 @@
         <v>2</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>1.14</v>
+        <v>1.13</v>
       </c>
       <c r="E13" s="5" t="n">
         <v>84454</v>
@@ -865,16 +865,16 @@
         <v>13</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>5.71</v>
+        <v>9.04</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>13135</v>
+        <v>11280</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>8758</v>
+        <v>8552</v>
       </c>
       <c r="G14" s="5" t="n">
         <v>7752</v>
@@ -891,16 +891,16 @@
         <v>14</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>2.86</v>
+        <v>5.65</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>8566</v>
+        <v>8403</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>8522</v>
+        <v>8224</v>
       </c>
       <c r="G15" s="5" t="n">
         <v>7752</v>
@@ -917,19 +917,19 @@
         <v>15</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>1.14</v>
+        <v>1.69</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>10462</v>
+        <v>9617</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>10462</v>
+        <v>8582</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>8582</v>
+        <v>7928</v>
       </c>
       <c r="H16" s="5" t="n">
         <v>12342</v>
@@ -946,7 +946,7 @@
         <v>3</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>1.71</v>
+        <v>1.69</v>
       </c>
       <c r="E17" s="5" t="n">
         <v>22533</v>
@@ -969,16 +969,16 @@
         <v>17</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>23.43</v>
+        <v>22.03</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>76586</v>
+        <v>79769</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>29242</v>
+        <v>40072</v>
       </c>
       <c r="G18" s="5" t="n">
         <v>8098</v>

</xml_diff>